<commit_message>
Add formatted Excel report, README and final screenshots
</commit_message>
<xml_diff>
--- a/data/cleaned_sales.xlsx
+++ b/data/cleaned_sales.xlsx
@@ -604,7 +604,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46362</v>
+        <v>46185</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1474,7 +1474,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46236</v>
+        <v>46061</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46027</v>
+        <v>46143</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46359</v>
+        <v>46093</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -2170,7 +2170,7 @@
     </row>
     <row r="61">
       <c r="A61" s="1" t="n">
-        <v>46175</v>
+        <v>46059</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
@@ -2286,7 +2286,7 @@
     </row>
     <row r="65">
       <c r="A65" s="1" t="n">
-        <v>45912</v>
+        <v>46000</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
     </row>
     <row r="66">
       <c r="A66" s="1" t="n">
-        <v>46236</v>
+        <v>46061</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -3156,7 +3156,7 @@
     </row>
     <row r="95">
       <c r="A95" s="1" t="n">
-        <v>45908</v>
+        <v>45878</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -3185,7 +3185,7 @@
     </row>
     <row r="96">
       <c r="A96" s="1" t="n">
-        <v>46145</v>
+        <v>46086</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -3243,7 +3243,7 @@
     </row>
     <row r="98">
       <c r="A98" s="1" t="n">
-        <v>46174</v>
+        <v>46028</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -3910,7 +3910,7 @@
     </row>
     <row r="121">
       <c r="A121" s="1" t="n">
-        <v>45756</v>
+        <v>45904</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -3939,7 +3939,7 @@
     </row>
     <row r="122">
       <c r="A122" s="1" t="n">
-        <v>46056</v>
+        <v>46083</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
@@ -4026,7 +4026,7 @@
     </row>
     <row r="125">
       <c r="A125" s="1" t="n">
-        <v>45668</v>
+        <v>45962</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
     </row>
     <row r="130">
       <c r="A130" s="1" t="n">
-        <v>45788</v>
+        <v>45966</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -4606,7 +4606,7 @@
     </row>
     <row r="145">
       <c r="A145" s="1" t="n">
-        <v>45848</v>
+        <v>45937</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -5186,7 +5186,7 @@
     </row>
     <row r="165">
       <c r="A165" s="1" t="n">
-        <v>46357</v>
+        <v>46034</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
@@ -5244,7 +5244,7 @@
     </row>
     <row r="167">
       <c r="A167" s="1" t="n">
-        <v>46297</v>
+        <v>46063</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -5418,7 +5418,7 @@
     </row>
     <row r="173">
       <c r="A173" s="1" t="n">
-        <v>46149</v>
+        <v>46208</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
@@ -5447,7 +5447,7 @@
     </row>
     <row r="174">
       <c r="A174" s="1" t="n">
-        <v>46054</v>
+        <v>46024</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -5911,7 +5911,7 @@
     </row>
     <row r="190">
       <c r="A190" s="1" t="n">
-        <v>46174</v>
+        <v>46028</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -6636,7 +6636,7 @@
     </row>
     <row r="215">
       <c r="A215" s="1" t="n">
-        <v>45697</v>
+        <v>45902</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
     </row>
     <row r="237">
       <c r="A237" s="1" t="n">
-        <v>46206</v>
+        <v>46088</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
@@ -7506,7 +7506,7 @@
     </row>
     <row r="245">
       <c r="A245" s="1" t="n">
-        <v>46267</v>
+        <v>46062</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
@@ -7883,7 +7883,7 @@
     </row>
     <row r="258">
       <c r="A258" s="1" t="n">
-        <v>46085</v>
+        <v>46115</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -8492,7 +8492,7 @@
     </row>
     <row r="279">
       <c r="A279" s="1" t="n">
-        <v>46270</v>
+        <v>46151</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
@@ -9072,7 +9072,7 @@
     </row>
     <row r="299">
       <c r="A299" s="1" t="n">
-        <v>46297</v>
+        <v>46063</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
@@ -9217,7 +9217,7 @@
     </row>
     <row r="304">
       <c r="A304" s="1" t="n">
-        <v>46114</v>
+        <v>46057</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
@@ -9652,7 +9652,7 @@
     </row>
     <row r="319">
       <c r="A319" s="1" t="n">
-        <v>46299</v>
+        <v>46122</v>
       </c>
       <c r="B319" t="inlineStr">
         <is>
@@ -9971,7 +9971,7 @@
     </row>
     <row r="330">
       <c r="A330" s="1" t="n">
-        <v>46208</v>
+        <v>46149</v>
       </c>
       <c r="B330" t="inlineStr">
         <is>
@@ -10145,7 +10145,7 @@
     </row>
     <row r="336">
       <c r="A336" s="1" t="n">
-        <v>46086</v>
+        <v>46145</v>
       </c>
       <c r="B336" t="inlineStr">
         <is>
@@ -10464,7 +10464,7 @@
     </row>
     <row r="347">
       <c r="A347" s="1" t="n">
-        <v>45820</v>
+        <v>45997</v>
       </c>
       <c r="B347" t="inlineStr">
         <is>
@@ -10522,7 +10522,7 @@
     </row>
     <row r="349">
       <c r="A349" s="1" t="n">
-        <v>46001</v>
+        <v>45942</v>
       </c>
       <c r="B349" t="inlineStr">
         <is>
@@ -10580,7 +10580,7 @@
     </row>
     <row r="351">
       <c r="A351" s="1" t="n">
-        <v>46149</v>
+        <v>46208</v>
       </c>
       <c r="B351" t="inlineStr">
         <is>
@@ -10638,7 +10638,7 @@
     </row>
     <row r="353">
       <c r="A353" s="1" t="n">
-        <v>45756</v>
+        <v>45904</v>
       </c>
       <c r="B353" t="inlineStr">
         <is>
@@ -11131,7 +11131,7 @@
     </row>
     <row r="370">
       <c r="A370" s="1" t="n">
-        <v>46028</v>
+        <v>46174</v>
       </c>
       <c r="B370" t="inlineStr">
         <is>
@@ -11247,7 +11247,7 @@
     </row>
     <row r="374">
       <c r="A374" s="1" t="n">
-        <v>45880</v>
+        <v>45969</v>
       </c>
       <c r="B374" t="inlineStr">
         <is>
@@ -11508,7 +11508,7 @@
     </row>
     <row r="383">
       <c r="A383" s="1" t="n">
-        <v>45817</v>
+        <v>45906</v>
       </c>
       <c r="B383" t="inlineStr">
         <is>
@@ -11653,7 +11653,7 @@
     </row>
     <row r="388">
       <c r="A388" s="1" t="n">
-        <v>46057</v>
+        <v>46114</v>
       </c>
       <c r="B388" t="inlineStr">
         <is>
@@ -11885,7 +11885,7 @@
     </row>
     <row r="396">
       <c r="A396" s="1" t="n">
-        <v>46083</v>
+        <v>46056</v>
       </c>
       <c r="B396" t="inlineStr">
         <is>
@@ -12088,7 +12088,7 @@
     </row>
     <row r="403">
       <c r="A403" s="1" t="n">
-        <v>46241</v>
+        <v>46211</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
@@ -12813,7 +12813,7 @@
     </row>
     <row r="428">
       <c r="A428" s="1" t="n">
-        <v>45971</v>
+        <v>45941</v>
       </c>
       <c r="B428" t="inlineStr">
         <is>
@@ -12958,7 +12958,7 @@
     </row>
     <row r="433">
       <c r="A433" s="1" t="n">
-        <v>46208</v>
+        <v>46149</v>
       </c>
       <c r="B433" t="inlineStr">
         <is>
@@ -13306,7 +13306,7 @@
     </row>
     <row r="445">
       <c r="A445" s="1" t="n">
-        <v>45757</v>
+        <v>45934</v>
       </c>
       <c r="B445" t="inlineStr">
         <is>
@@ -13799,7 +13799,7 @@
     </row>
     <row r="462">
       <c r="A462" s="1" t="n">
-        <v>46059</v>
+        <v>46175</v>
       </c>
       <c r="B462" t="inlineStr">
         <is>
@@ -13828,7 +13828,7 @@
     </row>
     <row r="463">
       <c r="A463" s="1" t="n">
-        <v>45848</v>
+        <v>45937</v>
       </c>
       <c r="B463" t="inlineStr">
         <is>
@@ -13857,7 +13857,7 @@
     </row>
     <row r="464">
       <c r="A464" s="1" t="n">
-        <v>45785</v>
+        <v>45874</v>
       </c>
       <c r="B464" t="inlineStr">
         <is>
@@ -13944,7 +13944,7 @@
     </row>
     <row r="467">
       <c r="A467" s="1" t="n">
-        <v>45910</v>
+        <v>45939</v>
       </c>
       <c r="B467" t="inlineStr">
         <is>
@@ -14234,7 +14234,7 @@
     </row>
     <row r="477">
       <c r="A477" s="1" t="n">
-        <v>45941</v>
+        <v>45971</v>
       </c>
       <c r="B477" t="inlineStr">
         <is>
@@ -14350,7 +14350,7 @@
     </row>
     <row r="481">
       <c r="A481" s="1" t="n">
-        <v>46361</v>
+        <v>46154</v>
       </c>
       <c r="B481" t="inlineStr">
         <is>
@@ -14437,7 +14437,7 @@
     </row>
     <row r="484">
       <c r="A484" s="1" t="n">
-        <v>46000</v>
+        <v>45912</v>
       </c>
       <c r="B484" t="inlineStr">
         <is>
@@ -14466,7 +14466,7 @@
     </row>
     <row r="485">
       <c r="A485" s="1" t="n">
-        <v>46236</v>
+        <v>46061</v>
       </c>
       <c r="B485" t="inlineStr">
         <is>
@@ -14553,7 +14553,7 @@
     </row>
     <row r="488">
       <c r="A488" s="1" t="n">
-        <v>45787</v>
+        <v>45935</v>
       </c>
       <c r="B488" t="inlineStr">
         <is>
@@ -14727,7 +14727,7 @@
     </row>
     <row r="494">
       <c r="A494" s="1" t="n">
-        <v>46207</v>
+        <v>46119</v>
       </c>
       <c r="B494" t="inlineStr">
         <is>
@@ -14814,7 +14814,7 @@
     </row>
     <row r="497">
       <c r="A497" s="1" t="n">
-        <v>46146</v>
+        <v>46117</v>
       </c>
       <c r="B497" t="inlineStr">
         <is>
@@ -14901,7 +14901,7 @@
     </row>
     <row r="500">
       <c r="A500" s="1" t="n">
-        <v>46114</v>
+        <v>46057</v>
       </c>
       <c r="B500" t="inlineStr">
         <is>
@@ -14930,7 +14930,7 @@
     </row>
     <row r="501">
       <c r="A501" s="1" t="n">
-        <v>46328</v>
+        <v>46064</v>
       </c>
       <c r="B501" t="inlineStr">
         <is>
@@ -15452,7 +15452,7 @@
     </row>
     <row r="519">
       <c r="A519" s="1" t="n">
-        <v>45908</v>
+        <v>45878</v>
       </c>
       <c r="B519" t="inlineStr">
         <is>
@@ -16235,7 +16235,7 @@
     </row>
     <row r="546">
       <c r="A546" s="1" t="n">
-        <v>46144</v>
+        <v>46058</v>
       </c>
       <c r="B546" t="inlineStr">
         <is>
@@ -16351,7 +16351,7 @@
     </row>
     <row r="550">
       <c r="A550" s="1" t="n">
-        <v>45787</v>
+        <v>45935</v>
       </c>
       <c r="B550" t="inlineStr">
         <is>
@@ -16931,7 +16931,7 @@
     </row>
     <row r="570">
       <c r="A570" s="1" t="n">
-        <v>46113</v>
+        <v>46026</v>
       </c>
       <c r="B570" t="inlineStr">
         <is>
@@ -17424,7 +17424,7 @@
     </row>
     <row r="587">
       <c r="A587" s="1" t="n">
-        <v>46241</v>
+        <v>46211</v>
       </c>
       <c r="B587" t="inlineStr">
         <is>
@@ -17540,7 +17540,7 @@
     </row>
     <row r="591">
       <c r="A591" s="1" t="n">
-        <v>46059</v>
+        <v>46175</v>
       </c>
       <c r="B591" t="inlineStr">
         <is>
@@ -17598,7 +17598,7 @@
     </row>
     <row r="593">
       <c r="A593" s="1" t="n">
-        <v>46143</v>
+        <v>46027</v>
       </c>
       <c r="B593" t="inlineStr">
         <is>
@@ -18178,7 +18178,7 @@
     </row>
     <row r="613">
       <c r="A613" s="1" t="n">
-        <v>45700</v>
+        <v>45993</v>
       </c>
       <c r="B613" t="inlineStr">
         <is>
@@ -18410,7 +18410,7 @@
     </row>
     <row r="621">
       <c r="A621" s="1" t="n">
-        <v>45846</v>
+        <v>45876</v>
       </c>
       <c r="B621" t="inlineStr">
         <is>
@@ -18439,7 +18439,7 @@
     </row>
     <row r="622">
       <c r="A622" s="1" t="n">
-        <v>45849</v>
+        <v>45968</v>
       </c>
       <c r="B622" t="inlineStr">
         <is>
@@ -18729,7 +18729,7 @@
     </row>
     <row r="632">
       <c r="A632" s="1" t="n">
-        <v>45666</v>
+        <v>45901</v>
       </c>
       <c r="B632" t="inlineStr">
         <is>
@@ -18758,7 +18758,7 @@
     </row>
     <row r="633">
       <c r="A633" s="1" t="n">
-        <v>46029</v>
+        <v>46204</v>
       </c>
       <c r="B633" t="inlineStr">
         <is>
@@ -18787,7 +18787,7 @@
     </row>
     <row r="634">
       <c r="A634" s="1" t="n">
-        <v>46359</v>
+        <v>46093</v>
       </c>
       <c r="B634" t="inlineStr">
         <is>
@@ -18845,7 +18845,7 @@
     </row>
     <row r="636">
       <c r="A636" s="1" t="n">
-        <v>46059</v>
+        <v>46175</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
@@ -19425,7 +19425,7 @@
     </row>
     <row r="656">
       <c r="A656" s="1" t="n">
-        <v>46209</v>
+        <v>46180</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
@@ -19686,7 +19686,7 @@
     </row>
     <row r="665">
       <c r="A665" s="1" t="n">
-        <v>45818</v>
+        <v>45936</v>
       </c>
       <c r="B665" t="inlineStr">
         <is>
@@ -19889,7 +19889,7 @@
     </row>
     <row r="672">
       <c r="A672" s="1" t="n">
-        <v>46363</v>
+        <v>46215</v>
       </c>
       <c r="B672" t="inlineStr">
         <is>
@@ -20324,7 +20324,7 @@
     </row>
     <row r="687">
       <c r="A687" s="1" t="n">
-        <v>46145</v>
+        <v>46086</v>
       </c>
       <c r="B687" t="inlineStr">
         <is>
@@ -20556,7 +20556,7 @@
     </row>
     <row r="695">
       <c r="A695" s="1" t="n">
-        <v>46357</v>
+        <v>46034</v>
       </c>
       <c r="B695" t="inlineStr">
         <is>
@@ -20585,7 +20585,7 @@
     </row>
     <row r="696">
       <c r="A696" s="1" t="n">
-        <v>46266</v>
+        <v>46031</v>
       </c>
       <c r="B696" t="inlineStr">
         <is>
@@ -20759,7 +20759,7 @@
     </row>
     <row r="702">
       <c r="A702" s="1" t="n">
-        <v>45698</v>
+        <v>45932</v>
       </c>
       <c r="B702" t="inlineStr">
         <is>
@@ -21136,7 +21136,7 @@
     </row>
     <row r="715">
       <c r="A715" s="1" t="n">
-        <v>45938</v>
+        <v>45879</v>
       </c>
       <c r="B715" t="inlineStr">
         <is>
@@ -21281,7 +21281,7 @@
     </row>
     <row r="720">
       <c r="A720" s="1" t="n">
-        <v>46027</v>
+        <v>46143</v>
       </c>
       <c r="B720" t="inlineStr">
         <is>
@@ -21745,7 +21745,7 @@
     </row>
     <row r="736">
       <c r="A736" s="1" t="n">
-        <v>46267</v>
+        <v>46062</v>
       </c>
       <c r="B736" t="inlineStr">
         <is>
@@ -21803,7 +21803,7 @@
     </row>
     <row r="738">
       <c r="A738" s="1" t="n">
-        <v>45785</v>
+        <v>45874</v>
       </c>
       <c r="B738" t="inlineStr">
         <is>
@@ -22238,7 +22238,7 @@
     </row>
     <row r="753">
       <c r="A753" s="1" t="n">
-        <v>45786</v>
+        <v>45905</v>
       </c>
       <c r="B753" t="inlineStr">
         <is>
@@ -22470,7 +22470,7 @@
     </row>
     <row r="761">
       <c r="A761" s="1" t="n">
-        <v>46024</v>
+        <v>46054</v>
       </c>
       <c r="B761" t="inlineStr">
         <is>
@@ -22615,7 +22615,7 @@
     </row>
     <row r="766">
       <c r="A766" s="1" t="n">
-        <v>46002</v>
+        <v>45973</v>
       </c>
       <c r="B766" t="inlineStr">
         <is>
@@ -22702,7 +22702,7 @@
     </row>
     <row r="769">
       <c r="A769" s="1" t="n">
-        <v>46087</v>
+        <v>46176</v>
       </c>
       <c r="B769" t="inlineStr">
         <is>
@@ -23021,7 +23021,7 @@
     </row>
     <row r="780">
       <c r="A780" s="1" t="n">
-        <v>45665</v>
+        <v>45870</v>
       </c>
       <c r="B780" t="inlineStr">
         <is>
@@ -23195,7 +23195,7 @@
     </row>
     <row r="786">
       <c r="A786" s="1" t="n">
-        <v>45971</v>
+        <v>45941</v>
       </c>
       <c r="B786" t="inlineStr">
         <is>
@@ -23862,7 +23862,7 @@
     </row>
     <row r="809">
       <c r="A809" s="1" t="n">
-        <v>46359</v>
+        <v>46093</v>
       </c>
       <c r="B809" t="inlineStr">
         <is>
@@ -24326,7 +24326,7 @@
     </row>
     <row r="825">
       <c r="A825" s="1" t="n">
-        <v>45969</v>
+        <v>45880</v>
       </c>
       <c r="B825" t="inlineStr">
         <is>
@@ -24500,7 +24500,7 @@
     </row>
     <row r="831">
       <c r="A831" s="1" t="n">
-        <v>46302</v>
+        <v>46213</v>
       </c>
       <c r="B831" t="inlineStr">
         <is>
@@ -24848,7 +24848,7 @@
     </row>
     <row r="843">
       <c r="A843" s="1" t="n">
-        <v>45848</v>
+        <v>45937</v>
       </c>
       <c r="B843" t="inlineStr">
         <is>
@@ -25109,7 +25109,7 @@
     </row>
     <row r="852">
       <c r="A852" s="1" t="n">
-        <v>46361</v>
+        <v>46154</v>
       </c>
       <c r="B852" t="inlineStr">
         <is>
@@ -25457,7 +25457,7 @@
     </row>
     <row r="864">
       <c r="A864" s="1" t="n">
-        <v>45668</v>
+        <v>45962</v>
       </c>
       <c r="B864" t="inlineStr">
         <is>
@@ -25602,7 +25602,7 @@
     </row>
     <row r="869">
       <c r="A869" s="1" t="n">
-        <v>46240</v>
+        <v>46181</v>
       </c>
       <c r="B869" t="inlineStr">
         <is>
@@ -25689,7 +25689,7 @@
     </row>
     <row r="872">
       <c r="A872" s="1" t="n">
-        <v>45669</v>
+        <v>45992</v>
       </c>
       <c r="B872" t="inlineStr">
         <is>
@@ -25892,7 +25892,7 @@
     </row>
     <row r="879">
       <c r="A879" s="1" t="n">
-        <v>46026</v>
+        <v>46113</v>
       </c>
       <c r="B879" t="inlineStr">
         <is>
@@ -26008,7 +26008,7 @@
     </row>
     <row r="883">
       <c r="A883" s="1" t="n">
-        <v>46082</v>
+        <v>46025</v>
       </c>
       <c r="B883" t="inlineStr">
         <is>
@@ -26501,7 +26501,7 @@
     </row>
     <row r="900">
       <c r="A900" s="1" t="n">
-        <v>46145</v>
+        <v>46086</v>
       </c>
       <c r="B900" t="inlineStr">
         <is>
@@ -26878,7 +26878,7 @@
     </row>
     <row r="913">
       <c r="A913" s="1" t="n">
-        <v>45881</v>
+        <v>45999</v>
       </c>
       <c r="B913" t="inlineStr">
         <is>
@@ -27168,7 +27168,7 @@
     </row>
     <row r="923">
       <c r="A923" s="1" t="n">
-        <v>46328</v>
+        <v>46064</v>
       </c>
       <c r="B923" t="inlineStr">
         <is>
@@ -27226,7 +27226,7 @@
     </row>
     <row r="925">
       <c r="A925" s="1" t="n">
-        <v>45879</v>
+        <v>45938</v>
       </c>
       <c r="B925" t="inlineStr">
         <is>
@@ -27371,7 +27371,7 @@
     </row>
     <row r="930">
       <c r="A930" s="1" t="n">
-        <v>46236</v>
+        <v>46061</v>
       </c>
       <c r="B930" t="inlineStr">
         <is>
@@ -27516,7 +27516,7 @@
     </row>
     <row r="935">
       <c r="A935" s="1" t="n">
-        <v>45970</v>
+        <v>45911</v>
       </c>
       <c r="B935" t="inlineStr">
         <is>
@@ -27806,7 +27806,7 @@
     </row>
     <row r="945">
       <c r="A945" s="1" t="n">
-        <v>45817</v>
+        <v>45906</v>
       </c>
       <c r="B945" t="inlineStr">
         <is>
@@ -28067,7 +28067,7 @@
     </row>
     <row r="954">
       <c r="A954" s="1" t="n">
-        <v>45847</v>
+        <v>45907</v>
       </c>
       <c r="B954" t="inlineStr">
         <is>
@@ -28299,7 +28299,7 @@
     </row>
     <row r="962">
       <c r="A962" s="1" t="n">
-        <v>45912</v>
+        <v>46000</v>
       </c>
       <c r="B962" t="inlineStr">
         <is>
@@ -28386,7 +28386,7 @@
     </row>
     <row r="965">
       <c r="A965" s="1" t="n">
-        <v>46056</v>
+        <v>46083</v>
       </c>
       <c r="B965" t="inlineStr">
         <is>
@@ -28473,7 +28473,7 @@
     </row>
     <row r="968">
       <c r="A968" s="1" t="n">
-        <v>46058</v>
+        <v>46144</v>
       </c>
       <c r="B968" t="inlineStr">
         <is>
@@ -28531,7 +28531,7 @@
     </row>
     <row r="970">
       <c r="A970" s="1" t="n">
-        <v>46027</v>
+        <v>46143</v>
       </c>
       <c r="B970" t="inlineStr">
         <is>
@@ -28618,7 +28618,7 @@
     </row>
     <row r="973">
       <c r="A973" s="1" t="n">
-        <v>46272</v>
+        <v>46212</v>
       </c>
       <c r="B973" t="inlineStr">
         <is>
@@ -28821,7 +28821,7 @@
     </row>
     <row r="980">
       <c r="A980" s="1" t="n">
-        <v>46056</v>
+        <v>46083</v>
       </c>
       <c r="B980" t="inlineStr">
         <is>
@@ -29314,7 +29314,7 @@
     </row>
     <row r="997">
       <c r="A997" s="1" t="n">
-        <v>46058</v>
+        <v>46144</v>
       </c>
       <c r="B997" t="inlineStr">
         <is>
@@ -29430,7 +29430,7 @@
     </row>
     <row r="1001">
       <c r="A1001" s="1" t="n">
-        <v>45785</v>
+        <v>45874</v>
       </c>
       <c r="B1001" t="inlineStr">
         <is>

</xml_diff>